<commit_message>
Add student profiles, Excel backup, import validation, and hosting build.
Introduce student_id-based import/export with calendar and cross-sheet validation, a school admin backup page matching the import template, student profile views with status logic, Supabase SSL fixes, and a standalone hosting-build packaging script.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/fwis-school-data-import-template.xlsx
+++ b/templates/fwis-school-data-import-template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="114">
   <si>
     <t>FWIS School Data Import Template</t>
   </si>
@@ -67,13 +67,19 @@
     <t xml:space="preserve">  • academic_year on Students/Attendance/Assessments must match School_Setup</t>
   </si>
   <si>
-    <t xml:space="preserve">  • grade: 1–6 or Grade 1 … Grade 6 on Teachers, Students, Attendance, Assessments</t>
+    <t xml:space="preserve">  • student_id: HOU-B1 (city code + B/G + number). Assign on Students first, then copy to Attendance/Assessments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • student_id on Students is optional — leave blank to auto-assign on import</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • grade: 1–6 or Grade 1 … Grade 6 on Teachers and Students</t>
   </si>
   <si>
     <t xml:space="preserve">  • section: Boys or Girls (exact capitalization recommended)</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Attendance/Assessments: grade + section must match the Students row for that child</t>
+    <t xml:space="preserve">  • Attendance/Assessments: use student_id from the Students sheet (must match exactly)</t>
   </si>
   <si>
     <t xml:space="preserve">  • gender: MALE or FEMALE (MALE→Boys, FEMALE→Girls)</t>
@@ -88,6 +94,15 @@
     <t xml:space="preserve">  • status: Present, Absent, or Tardy</t>
   </si>
   <si>
+    <t xml:space="preserve">  • Calendar_Optional: mark HOLIDAY, QUIZ_1–QUIZ_5, FINAL_EXAM, etc. per Sunday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Do not record attendance on HOLIDAY, PARENT_MEETING, or GRADUATION days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Quiz and final exam days on the calendar require matching scores on Assessments</t>
+  </si>
+  <si>
     <t xml:space="preserve">  • assessment scores: 0–100; leave blank if not taken</t>
   </si>
   <si>
@@ -166,7 +181,7 @@
     <t>Usman Khan</t>
   </si>
   <si>
-    <t>teacher.grade1.boys.houston@fwis.org</t>
+    <t>grade1.boys.houston@fwis.org</t>
   </si>
   <si>
     <t>555-3001</t>
@@ -184,7 +199,7 @@
     <t>Ali Khan</t>
   </si>
   <si>
-    <t>teacher.grade1.girls.houston@fwis.org</t>
+    <t>grade1.girls.houston@fwis.org</t>
   </si>
   <si>
     <t>555-3002</t>
@@ -193,6 +208,9 @@
     <t>Girls</t>
   </si>
   <si>
+    <t>student_id</t>
+  </si>
+  <si>
     <t>gender</t>
   </si>
   <si>
@@ -211,6 +229,9 @@
     <t>enrollment_date</t>
   </si>
   <si>
+    <t>HOU-B1</t>
+  </si>
+  <si>
     <t>Ahmed</t>
   </si>
   <si>
@@ -229,6 +250,9 @@
     <t>parent.khan@email.com</t>
   </si>
   <si>
+    <t>HOU-G1</t>
+  </si>
+  <si>
     <t>Aisha</t>
   </si>
   <si>
@@ -247,12 +271,6 @@
     <t>parent.ali@email.com</t>
   </si>
   <si>
-    <t>student_first_name</t>
-  </si>
-  <si>
-    <t>student_last_name</t>
-  </si>
-  <si>
     <t>date</t>
   </si>
   <si>
@@ -337,7 +355,7 @@
     <t>2024-10-06</t>
   </si>
   <si>
-    <t>QUIZ</t>
+    <t>QUIZ_1</t>
   </si>
   <si>
     <t>5</t>
@@ -734,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -882,12 +900,37 @@
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -906,42 +949,42 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -960,80 +1003,80 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="H2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" t="s">
         <v>56</v>
       </c>
-      <c r="G3" t="s">
-        <v>51</v>
-      </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1043,273 +1086,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="13" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" t="s">
-        <v>66</v>
-      </c>
-      <c r="G2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H2" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" t="s">
-        <v>49</v>
-      </c>
-      <c r="J2" t="s">
-        <v>67</v>
-      </c>
-      <c r="K2" t="s">
-        <v>68</v>
-      </c>
-      <c r="L2" t="s">
-        <v>69</v>
-      </c>
-      <c r="M2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" t="s">
-        <v>71</v>
-      </c>
-      <c r="F3" t="s">
-        <v>72</v>
-      </c>
-      <c r="G3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" t="s">
-        <v>57</v>
-      </c>
-      <c r="I3" t="s">
-        <v>55</v>
-      </c>
-      <c r="J3" t="s">
-        <v>73</v>
-      </c>
-      <c r="K3" t="s">
-        <v>74</v>
-      </c>
-      <c r="L3" t="s">
-        <v>75</v>
-      </c>
-      <c r="M3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="9" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" t="s">
-        <v>81</v>
-      </c>
-      <c r="I3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F4" t="s">
-        <v>51</v>
-      </c>
-      <c r="G4" t="s">
-        <v>57</v>
-      </c>
-      <c r="H4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1319,134 +1095,347 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="G2" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="H2" t="s">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="J2" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="K2" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="L2" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="M2" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="N2" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" t="s">
+        <v>60</v>
+      </c>
+      <c r="K3" t="s">
+        <v>81</v>
+      </c>
+      <c r="L3" t="s">
+        <v>82</v>
+      </c>
+      <c r="M3" t="s">
+        <v>83</v>
+      </c>
+      <c r="N3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>35</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
         <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="11" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" t="s">
+        <v>98</v>
+      </c>
+      <c r="H2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F3" t="s">
+        <v>104</v>
       </c>
       <c r="G3" t="s">
-        <v>57</v>
+        <v>105</v>
       </c>
       <c r="H3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I3" t="s">
+        <v>106</v>
+      </c>
+      <c r="J3" t="s">
         <v>98</v>
       </c>
-      <c r="J3" t="s">
-        <v>99</v>
-      </c>
       <c r="K3" t="s">
-        <v>90</v>
-      </c>
-      <c r="L3" t="s">
-        <v>100</v>
-      </c>
-      <c r="M3" t="s">
-        <v>92</v>
-      </c>
-      <c r="N3" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1467,46 +1456,46 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C4" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>